<commit_message>
2026C Q1 done, ready for Q2
</commit_message>
<xml_diff>
--- a/2026C_formal/outputs/result1.xlsx
+++ b/2026C_formal/outputs/result1.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="941" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="1259" uniqueCount="158">
   <si>
     <t>时间段</t>
   </si>
@@ -1106,7 +1106,7 @@
         <v>70</v>
       </c>
       <c r="B71" s="0">
-        <v>179.27717139917996</v>
+        <v>179.277171399178</v>
       </c>
     </row>
     <row r="72">
@@ -1114,7 +1114,7 @@
         <v>71</v>
       </c>
       <c r="B72" s="0">
-        <v>520.12451666666675</v>
+        <v>520.12451666666652</v>
       </c>
     </row>
     <row r="73">
@@ -1122,7 +1122,7 @@
         <v>72</v>
       </c>
       <c r="B73" s="0">
-        <v>486.4028999999997</v>
+        <v>486.40289999999987</v>
       </c>
     </row>
     <row r="74">
@@ -1130,7 +1130,7 @@
         <v>73</v>
       </c>
       <c r="B74" s="0">
-        <v>480.41244999999981</v>
+        <v>480.41244999999992</v>
       </c>
     </row>
     <row r="75">
@@ -1146,7 +1146,7 @@
         <v>75</v>
       </c>
       <c r="B76" s="0">
-        <v>488.60696666666627</v>
+        <v>488.60696666666655</v>
       </c>
     </row>
     <row r="77">
@@ -1666,7 +1666,7 @@
         <v>140</v>
       </c>
       <c r="B141" s="0">
-        <v>569.35863333333555</v>
+        <v>569.35863333333327</v>
       </c>
     </row>
     <row r="142">
@@ -1682,7 +1682,7 @@
         <v>142</v>
       </c>
       <c r="B143" s="0">
-        <v>904.94871666666461</v>
+        <v>904.94871666666688</v>
       </c>
     </row>
     <row r="144">
@@ -1773,7 +1773,7 @@
         <v>148</v>
       </c>
       <c r="B4" s="0">
-        <v>4787.9642880658466</v>
+        <v>4787.9642880658439</v>
       </c>
       <c r="C4" s="0">
         <v>1702.9969833333332</v>
@@ -1812,7 +1812,7 @@
         <v>151</v>
       </c>
       <c r="B7" s="0">
-        <v>5333.3333333333303</v>
+        <v>5333.3333333333321</v>
       </c>
       <c r="C7" s="0">
         <v>2859.8681166666665</v>

</xml_diff>

<commit_message>
2026C  Q2 done, ready for Q3
</commit_message>
<xml_diff>
--- a/2026C_formal/outputs/result1.xlsx
+++ b/2026C_formal/outputs/result1.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="1259" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="1577" uniqueCount="158">
   <si>
     <t>时间段</t>
   </si>
@@ -554,7 +554,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="0">
-        <v>1406.6411000000001</v>
+        <v>907.4543166666665</v>
       </c>
     </row>
     <row r="3">
@@ -562,7 +562,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="0">
-        <v>1406.3298666666665</v>
+        <v>1406.6411000000001</v>
       </c>
     </row>
     <row r="4">
@@ -570,7 +570,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="0">
-        <v>1407.3838500000002</v>
+        <v>1406.3298666666665</v>
       </c>
     </row>
     <row r="5">
@@ -578,7 +578,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="0">
-        <v>1409.07395</v>
+        <v>1407.3838500000002</v>
       </c>
     </row>
     <row r="6">
@@ -586,7 +586,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="0">
-        <v>1409.8045500000001</v>
+        <v>1409.07395</v>
       </c>
     </row>
     <row r="7">
@@ -594,7 +594,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="0">
-        <v>576.64001666666661</v>
+        <v>1409.8045500000001</v>
       </c>
     </row>
     <row r="8">
@@ -602,7 +602,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="0">
-        <v>577.85969999999998</v>
+        <v>576.64001666666661</v>
       </c>
     </row>
     <row r="9">
@@ -610,7 +610,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="0">
-        <v>577.99386666666669</v>
+        <v>577.85969999999998</v>
       </c>
     </row>
     <row r="10">
@@ -618,7 +618,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="0">
-        <v>911.16138333333333</v>
+        <v>577.99386666666669</v>
       </c>
     </row>
     <row r="11">
@@ -626,7 +626,7 @@
         <v>10</v>
       </c>
       <c r="B11" s="0">
-        <v>580.41544999999997</v>
+        <v>577.82804999999996</v>
       </c>
     </row>
     <row r="12">
@@ -634,7 +634,7 @@
         <v>11</v>
       </c>
       <c r="B12" s="0">
-        <v>582.51401666666663</v>
+        <v>580.41544999999997</v>
       </c>
     </row>
     <row r="13">
@@ -642,7 +642,7 @@
         <v>12</v>
       </c>
       <c r="B13" s="0">
-        <v>583.07404999999994</v>
+        <v>582.51401666666663</v>
       </c>
     </row>
     <row r="14">
@@ -650,7 +650,7 @@
         <v>13</v>
       </c>
       <c r="B14" s="0">
-        <v>584.20491666666658</v>
+        <v>583.07404999999994</v>
       </c>
     </row>
     <row r="15">
@@ -658,7 +658,7 @@
         <v>14</v>
       </c>
       <c r="B15" s="0">
-        <v>585.43978333333325</v>
+        <v>584.20491666666658</v>
       </c>
     </row>
     <row r="16">
@@ -666,7 +666,7 @@
         <v>15</v>
       </c>
       <c r="B16" s="0">
-        <v>586.14474999999993</v>
+        <v>585.43978333333325</v>
       </c>
     </row>
     <row r="17">
@@ -674,7 +674,7 @@
         <v>16</v>
       </c>
       <c r="B17" s="0">
-        <v>586.3207666666666</v>
+        <v>586.14474999999993</v>
       </c>
     </row>
     <row r="18">
@@ -682,7 +682,7 @@
         <v>17</v>
       </c>
       <c r="B18" s="0">
-        <v>586.42529999999999</v>
+        <v>586.3207666666666</v>
       </c>
     </row>
     <row r="19">
@@ -690,7 +690,7 @@
         <v>18</v>
       </c>
       <c r="B19" s="0">
-        <v>586.84960000000001</v>
+        <v>586.42529999999999</v>
       </c>
     </row>
     <row r="20">
@@ -698,7 +698,7 @@
         <v>19</v>
       </c>
       <c r="B20" s="0">
-        <v>587.82101666666665</v>
+        <v>586.84960000000001</v>
       </c>
     </row>
     <row r="21">
@@ -706,7 +706,7 @@
         <v>20</v>
       </c>
       <c r="B21" s="0">
-        <v>589.54756666666663</v>
+        <v>587.82101666666665</v>
       </c>
     </row>
     <row r="22">
@@ -714,7 +714,7 @@
         <v>21</v>
       </c>
       <c r="B22" s="0">
-        <v>590.81346666666661</v>
+        <v>589.54756666666663</v>
       </c>
     </row>
     <row r="23">
@@ -722,7 +722,7 @@
         <v>22</v>
       </c>
       <c r="B23" s="0">
-        <v>590.21311666666657</v>
+        <v>590.81346666666661</v>
       </c>
     </row>
     <row r="24">
@@ -730,7 +730,7 @@
         <v>23</v>
       </c>
       <c r="B24" s="0">
-        <v>591.06626666666659</v>
+        <v>590.21311666666657</v>
       </c>
     </row>
     <row r="25">
@@ -738,7 +738,7 @@
         <v>24</v>
       </c>
       <c r="B25" s="0">
-        <v>593.36783333333324</v>
+        <v>591.06626666666659</v>
       </c>
     </row>
     <row r="26">
@@ -746,7 +746,7 @@
         <v>25</v>
       </c>
       <c r="B26" s="0">
-        <v>593.65968333333331</v>
+        <v>593.36783333333324</v>
       </c>
     </row>
     <row r="27">
@@ -754,7 +754,7 @@
         <v>26</v>
       </c>
       <c r="B27" s="0">
-        <v>592.78638333333333</v>
+        <v>593.65968333333331</v>
       </c>
     </row>
     <row r="28">
@@ -762,7 +762,7 @@
         <v>27</v>
       </c>
       <c r="B28" s="0">
-        <v>593.33786666666663</v>
+        <v>592.78638333333333</v>
       </c>
     </row>
     <row r="29">
@@ -770,7 +770,7 @@
         <v>28</v>
       </c>
       <c r="B29" s="0">
-        <v>596.67576666666662</v>
+        <v>593.33786666666663</v>
       </c>
     </row>
     <row r="30">
@@ -778,7 +778,7 @@
         <v>29</v>
       </c>
       <c r="B30" s="0">
-        <v>597.78025000000002</v>
+        <v>596.67576666666662</v>
       </c>
     </row>
     <row r="31">
@@ -786,7 +786,7 @@
         <v>30</v>
       </c>
       <c r="B31" s="0">
-        <v>595.16249999999991</v>
+        <v>597.78025000000002</v>
       </c>
     </row>
     <row r="32">
@@ -794,7 +794,7 @@
         <v>31</v>
       </c>
       <c r="B32" s="0">
-        <v>590.60649999999998</v>
+        <v>595.16249999999991</v>
       </c>
     </row>
     <row r="33">
@@ -802,7 +802,7 @@
         <v>32</v>
       </c>
       <c r="B33" s="0">
-        <v>589.48518333333334</v>
+        <v>590.60649999999998</v>
       </c>
     </row>
     <row r="34">
@@ -810,7 +810,7 @@
         <v>33</v>
       </c>
       <c r="B34" s="0">
-        <v>578.45544999999993</v>
+        <v>589.48518333333334</v>
       </c>
     </row>
     <row r="35">
@@ -818,7 +818,7 @@
         <v>34</v>
       </c>
       <c r="B35" s="0">
-        <v>1383.6597833333331</v>
+        <v>578.45544999999993</v>
       </c>
     </row>
     <row r="36">
@@ -826,7 +826,7 @@
         <v>35</v>
       </c>
       <c r="B36" s="0">
-        <v>591.14019999999994</v>
+        <v>1383.6597833333331</v>
       </c>
     </row>
     <row r="37">
@@ -834,7 +834,7 @@
         <v>36</v>
       </c>
       <c r="B37" s="0">
-        <v>0</v>
+        <v>591.14019999999994</v>
       </c>
     </row>
     <row r="38">
@@ -1082,7 +1082,7 @@
         <v>67</v>
       </c>
       <c r="B68" s="0">
-        <v>575.17091666666659</v>
+        <v>0</v>
       </c>
     </row>
     <row r="69">
@@ -1090,7 +1090,7 @@
         <v>68</v>
       </c>
       <c r="B69" s="0">
-        <v>0</v>
+        <v>575.17091666666659</v>
       </c>
     </row>
     <row r="70">
@@ -1106,7 +1106,7 @@
         <v>70</v>
       </c>
       <c r="B71" s="0">
-        <v>179.277171399178</v>
+        <v>0</v>
       </c>
     </row>
     <row r="72">
@@ -1114,7 +1114,7 @@
         <v>71</v>
       </c>
       <c r="B72" s="0">
-        <v>520.12451666666652</v>
+        <v>179.277171399178</v>
       </c>
     </row>
     <row r="73">
@@ -1122,7 +1122,7 @@
         <v>72</v>
       </c>
       <c r="B73" s="0">
-        <v>486.40289999999987</v>
+        <v>520.12451666666652</v>
       </c>
     </row>
     <row r="74">
@@ -1130,7 +1130,7 @@
         <v>73</v>
       </c>
       <c r="B74" s="0">
-        <v>480.41244999999992</v>
+        <v>486.40289999999987</v>
       </c>
     </row>
     <row r="75">
@@ -1138,7 +1138,7 @@
         <v>74</v>
       </c>
       <c r="B75" s="0">
-        <v>485.30000000000001</v>
+        <v>480.41244999999992</v>
       </c>
     </row>
     <row r="76">
@@ -1146,7 +1146,7 @@
         <v>75</v>
       </c>
       <c r="B76" s="0">
-        <v>488.60696666666655</v>
+        <v>485.30000000000001</v>
       </c>
     </row>
     <row r="77">
@@ -1154,7 +1154,7 @@
         <v>76</v>
       </c>
       <c r="B77" s="0">
-        <v>498.27073333333328</v>
+        <v>488.60696666666655</v>
       </c>
     </row>
     <row r="78">
@@ -1162,7 +1162,7 @@
         <v>77</v>
       </c>
       <c r="B78" s="0">
-        <v>0</v>
+        <v>498.27073333333328</v>
       </c>
     </row>
     <row r="79">
@@ -1266,7 +1266,7 @@
         <v>90</v>
       </c>
       <c r="B91" s="0">
-        <v>112.08986666666669</v>
+        <v>0</v>
       </c>
     </row>
     <row r="92">
@@ -1274,7 +1274,7 @@
         <v>91</v>
       </c>
       <c r="B92" s="0">
-        <v>266.73269362139911</v>
+        <v>112.08986666666669</v>
       </c>
     </row>
     <row r="93">
@@ -1282,7 +1282,7 @@
         <v>92</v>
       </c>
       <c r="B93" s="0">
-        <v>197.52351666666664</v>
+        <v>266.73269362139911</v>
       </c>
     </row>
     <row r="94">
@@ -1290,7 +1290,7 @@
         <v>93</v>
       </c>
       <c r="B94" s="0">
-        <v>244.81403333333324</v>
+        <v>197.52351666666664</v>
       </c>
     </row>
     <row r="95">
@@ -1298,7 +1298,7 @@
         <v>94</v>
       </c>
       <c r="B95" s="0">
-        <v>295.53461666666669</v>
+        <v>244.81403333333324</v>
       </c>
     </row>
     <row r="96">
@@ -1306,7 +1306,7 @@
         <v>95</v>
       </c>
       <c r="B96" s="0">
-        <v>345.77750000000003</v>
+        <v>295.53461666666669</v>
       </c>
     </row>
     <row r="97">
@@ -1314,7 +1314,7 @@
         <v>96</v>
       </c>
       <c r="B97" s="0">
-        <v>394.93148333333335</v>
+        <v>345.77750000000003</v>
       </c>
     </row>
     <row r="98">
@@ -1322,7 +1322,7 @@
         <v>97</v>
       </c>
       <c r="B98" s="0">
-        <v>445.43165000000005</v>
+        <v>394.93148333333335</v>
       </c>
     </row>
     <row r="99">
@@ -1330,7 +1330,7 @@
         <v>98</v>
       </c>
       <c r="B99" s="0">
-        <v>495.69658333333325</v>
+        <v>445.43165000000005</v>
       </c>
     </row>
     <row r="100">
@@ -1338,7 +1338,7 @@
         <v>99</v>
       </c>
       <c r="B100" s="0">
-        <v>547.11905000000002</v>
+        <v>495.69658333333325</v>
       </c>
     </row>
     <row r="101">
@@ -1346,7 +1346,7 @@
         <v>100</v>
       </c>
       <c r="B101" s="0">
-        <v>599.98543333333328</v>
+        <v>547.11905000000002</v>
       </c>
     </row>
     <row r="102">
@@ -1354,7 +1354,7 @@
         <v>101</v>
       </c>
       <c r="B102" s="0">
-        <v>635.4297499999999</v>
+        <v>599.98543333333328</v>
       </c>
     </row>
     <row r="103">
@@ -1362,7 +1362,7 @@
         <v>102</v>
       </c>
       <c r="B103" s="0">
-        <v>660.83068333333336</v>
+        <v>635.4297499999999</v>
       </c>
     </row>
     <row r="104">
@@ -1370,7 +1370,7 @@
         <v>103</v>
       </c>
       <c r="B104" s="0">
-        <v>702.03693333333331</v>
+        <v>660.83068333333336</v>
       </c>
     </row>
     <row r="105">
@@ -1378,7 +1378,7 @@
         <v>104</v>
       </c>
       <c r="B105" s="0">
-        <v>738.06578333333323</v>
+        <v>702.03693333333331</v>
       </c>
     </row>
     <row r="106">
@@ -1386,7 +1386,7 @@
         <v>105</v>
       </c>
       <c r="B106" s="0">
-        <v>775.94471666666664</v>
+        <v>738.06578333333323</v>
       </c>
     </row>
     <row r="107">
@@ -1394,7 +1394,7 @@
         <v>106</v>
       </c>
       <c r="B107" s="0">
-        <v>826.08324999999991</v>
+        <v>775.94471666666664</v>
       </c>
     </row>
     <row r="108">
@@ -1402,7 +1402,7 @@
         <v>107</v>
       </c>
       <c r="B108" s="0">
-        <v>762.42279999999994</v>
+        <v>826.08324999999991</v>
       </c>
     </row>
     <row r="109">
@@ -1410,7 +1410,7 @@
         <v>108</v>
       </c>
       <c r="B109" s="0">
-        <v>636.98261666666667</v>
+        <v>762.42279999999994</v>
       </c>
     </row>
     <row r="110">
@@ -1418,7 +1418,7 @@
         <v>109</v>
       </c>
       <c r="B110" s="0">
-        <v>531.89404999999988</v>
+        <v>636.98261666666667</v>
       </c>
     </row>
     <row r="111">
@@ -1426,7 +1426,7 @@
         <v>110</v>
       </c>
       <c r="B111" s="0">
-        <v>678.83053333333328</v>
+        <v>531.89404999999988</v>
       </c>
     </row>
     <row r="112">
@@ -1434,7 +1434,7 @@
         <v>111</v>
       </c>
       <c r="B112" s="0">
-        <v>686.2684999999999</v>
+        <v>678.83053333333328</v>
       </c>
     </row>
     <row r="113">
@@ -1442,7 +1442,7 @@
         <v>112</v>
       </c>
       <c r="B113" s="0">
-        <v>696.50438333333318</v>
+        <v>686.2684999999999</v>
       </c>
     </row>
     <row r="114">
@@ -1450,7 +1450,7 @@
         <v>113</v>
       </c>
       <c r="B114" s="0">
-        <v>0</v>
+        <v>696.50438333333318</v>
       </c>
     </row>
     <row r="115">
@@ -1546,7 +1546,7 @@
         <v>125</v>
       </c>
       <c r="B126" s="0">
-        <v>715.86891666666657</v>
+        <v>0</v>
       </c>
     </row>
     <row r="127">
@@ -1554,7 +1554,7 @@
         <v>126</v>
       </c>
       <c r="B127" s="0">
-        <v>717.00511666666671</v>
+        <v>715.86891666666657</v>
       </c>
     </row>
     <row r="128">
@@ -1562,7 +1562,7 @@
         <v>127</v>
       </c>
       <c r="B128" s="0">
-        <v>720.16030000000001</v>
+        <v>717.00511666666671</v>
       </c>
     </row>
     <row r="129">
@@ -1570,7 +1570,7 @@
         <v>128</v>
       </c>
       <c r="B129" s="0">
-        <v>717.05486666666661</v>
+        <v>720.16030000000001</v>
       </c>
     </row>
     <row r="130">
@@ -1578,7 +1578,7 @@
         <v>129</v>
       </c>
       <c r="B130" s="0">
-        <v>720.44596666666666</v>
+        <v>717.05486666666661</v>
       </c>
     </row>
     <row r="131">
@@ -1586,7 +1586,7 @@
         <v>130</v>
       </c>
       <c r="B131" s="0">
-        <v>738.13471666666658</v>
+        <v>720.44596666666666</v>
       </c>
     </row>
     <row r="132">
@@ -1594,7 +1594,7 @@
         <v>131</v>
       </c>
       <c r="B132" s="0">
-        <v>671.69356666666658</v>
+        <v>738.13471666666658</v>
       </c>
     </row>
     <row r="133">
@@ -1602,7 +1602,7 @@
         <v>132</v>
       </c>
       <c r="B133" s="0">
-        <v>1393.7903166666667</v>
+        <v>671.69356666666658</v>
       </c>
     </row>
     <row r="134">
@@ -1610,7 +1610,7 @@
         <v>133</v>
       </c>
       <c r="B134" s="0">
-        <v>1384.8989000000001</v>
+        <v>1393.7903166666667</v>
       </c>
     </row>
     <row r="135">
@@ -1618,7 +1618,7 @@
         <v>134</v>
       </c>
       <c r="B135" s="0">
-        <v>568.8260499999999</v>
+        <v>1384.8989000000001</v>
       </c>
     </row>
     <row r="136">
@@ -1626,7 +1626,7 @@
         <v>135</v>
       </c>
       <c r="B136" s="0">
-        <v>1396.98855</v>
+        <v>568.8260499999999</v>
       </c>
     </row>
     <row r="137">
@@ -1634,7 +1634,7 @@
         <v>136</v>
       </c>
       <c r="B137" s="0">
-        <v>1397.7598666666665</v>
+        <v>1396.98855</v>
       </c>
     </row>
     <row r="138">
@@ -1642,7 +1642,7 @@
         <v>137</v>
       </c>
       <c r="B138" s="0">
-        <v>566.74743333333322</v>
+        <v>1397.7598666666665</v>
       </c>
     </row>
     <row r="139">
@@ -1650,7 +1650,7 @@
         <v>138</v>
       </c>
       <c r="B139" s="0">
-        <v>1399.8737666666666</v>
+        <v>566.74743333333322</v>
       </c>
     </row>
     <row r="140">
@@ -1658,7 +1658,7 @@
         <v>139</v>
       </c>
       <c r="B140" s="0">
-        <v>567.83015</v>
+        <v>1399.8737666666666</v>
       </c>
     </row>
     <row r="141">
@@ -1666,7 +1666,7 @@
         <v>140</v>
       </c>
       <c r="B141" s="0">
-        <v>569.35863333333327</v>
+        <v>567.83015</v>
       </c>
     </row>
     <row r="142">
@@ -1674,7 +1674,7 @@
         <v>141</v>
       </c>
       <c r="B142" s="0">
-        <v>1403.6635166666667</v>
+        <v>902.69196666666653</v>
       </c>
     </row>
     <row r="143">
@@ -1682,7 +1682,7 @@
         <v>142</v>
       </c>
       <c r="B143" s="0">
-        <v>904.94871666666688</v>
+        <v>1403.6635166666667</v>
       </c>
     </row>
     <row r="144">
@@ -1690,7 +1690,7 @@
         <v>143</v>
       </c>
       <c r="B144" s="0">
-        <v>573.17683333333332</v>
+        <v>571.61538333333329</v>
       </c>
     </row>
     <row r="145">
@@ -1698,7 +1698,7 @@
         <v>144</v>
       </c>
       <c r="B145" s="0">
-        <v>574.12098333333324</v>
+        <v>573.17683333333332</v>
       </c>
     </row>
   </sheetData>
@@ -1759,7 +1759,7 @@
         <v>833.33333333333326</v>
       </c>
       <c r="C3" s="0">
-        <v>6365.8411999999999</v>
+        <v>5947.41975</v>
       </c>
       <c r="D3" s="0" t="s">
         <v>156</v>
@@ -1773,10 +1773,10 @@
         <v>148</v>
       </c>
       <c r="B4" s="0">
-        <v>4787.9642880658439</v>
+        <v>3954.6309547325109</v>
       </c>
       <c r="C4" s="0">
-        <v>1702.9969833333332</v>
+        <v>2121.4184333333328</v>
       </c>
       <c r="D4" s="0"/>
       <c r="E4" s="0"/>
@@ -1786,7 +1786,7 @@
         <v>149</v>
       </c>
       <c r="B5" s="0">
-        <v>5286.0351769547315</v>
+        <v>6119.3685102880654</v>
       </c>
       <c r="C5" s="0">
         <v>91.101383333333445</v>
@@ -1802,7 +1802,7 @@
         <v>0</v>
       </c>
       <c r="C6" s="0">
-        <v>5780.1318833333335</v>
+        <v>5068.68685</v>
       </c>
       <c r="D6" s="0"/>
       <c r="E6" s="0"/>
@@ -1815,7 +1815,7 @@
         <v>5333.3333333333321</v>
       </c>
       <c r="C7" s="0">
-        <v>2859.8681166666665</v>
+        <v>3571.31315</v>
       </c>
       <c r="D7" s="0"/>
       <c r="E7" s="0"/>

</xml_diff>